<commit_message>
updated useeio test and fixture
</commit_message>
<xml_diff>
--- a/tests/fixtures/databases/fixture_USEEIOv2.0.1-411.xlsx
+++ b/tests/fixtures/databases/fixture_USEEIOv2.0.1-411.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michaelweinold/github/GreenGraph/tests/fixtures/databases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA36976-CB0D-7045-ACF0-FBA96D529B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF19C306-F860-FC4F-B0E5-3C4B8523B8DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34560" yWindow="-8040" windowWidth="31800" windowHeight="23340" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34560" yWindow="500" windowWidth="31800" windowHeight="23340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="A" sheetId="4" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="70">
   <si>
     <t>1111A0/US</t>
   </si>
@@ -882,7 +882,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -947,6 +947,23 @@
         <v>0</v>
       </c>
       <c r="E4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
         <v>0</v>
       </c>
     </row>

</xml_diff>